<commit_message>
Simplificar presupuesto Juliana: sacar bolsas de provisiones y columna vigencia, notas solo con links de Drive
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Ruge_para_Juliana_30ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Ruge_para_Juliana_30ago2026.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Presupuesto para Juliana" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle contenido bolsas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -59,7 +58,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -68,7 +67,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,17 +432,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,15 +472,10 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Vigencia / fecha límite</t>
+          <t>Gestionado por</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Gestionado por</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -517,19 +509,10 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>⚠ Plazo original venció 27 ago — revalidar vigencia antes de aprobar</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
           <t>Marco Guanuchi</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Presupuesto Nº — recibido 28 ago</t>
-        </is>
-      </c>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -539,7 +522,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Talleres Fandos S.L. (Fandos Rent), Paterna</t>
+          <t>Talleres Fandos S.L. (Fandos Rent), Paterna — 638 81 96 48</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -554,22 +537,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Depósito 300€ + alquiler — confirmar forma de pago con Fandos (638 81 96 48)</t>
+          <t>Depósito 300€ + alquiler — confirmar forma de pago con Fandos</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Válido 10 días desde 25 ago — revisar si sigue vigente</t>
+          <t>David Luzuriaga</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>David Luzuriaga</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Presupuesto Nº 0325/26. PDF: Drive Mariano</t>
+          <t>https://drive.google.com/file/d/1wAsPjYeVI59B_aIMXqs-A4_4vj3f-t46/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -601,17 +579,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sin fecha límite en el presupuesto</t>
+          <t>Julio César Navia</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Julio César Navia</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>PDF: Drive Mariano</t>
+          <t>https://drive.google.com/file/d/1iK3L8s8NCgFfXymTNTYn1B94iH_TraiX/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -643,19 +616,10 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sin fecha límite en el presupuesto</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
           <t>Marco Guanuchi (a confirmar con Julio)</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>PLA, posprocesado y pintado incluido</t>
-        </is>
-      </c>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -665,7 +629,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Distribuciones Pascual, Catarroja</t>
+          <t>Distribuciones Pascual, Catarroja — Presupuesto Nº 2500004</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -685,19 +649,10 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto emitido 26 ago — revisar vigencia</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
           <t>David Luzuriaga</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Presupuesto Nº 2500004. Cubre el faltante de 43/90 redondeado a 50</t>
-        </is>
-      </c>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -707,7 +662,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Amazon — link B0DS2GM9QR</t>
+          <t>Amazon — https://www.amazon.es/dp/B0DS2GM9QR</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -727,19 +682,10 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
           <t>Marco Guanuchi</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Faltan 6 de 30 (hay 24)</t>
-        </is>
-      </c>
+      <c r="G7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -749,7 +695,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Amazon — link B0CQ2CWX1Y</t>
+          <t>Amazon — https://www.amazon.es/dp/B0CQ2CWX1Y</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -769,19 +715,10 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
           <t>Marco Guanuchi</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Marca NefLaca — hacen falta 90 en total, ya hay algunas en stock</t>
-        </is>
-      </c>
+      <c r="G8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -811,19 +748,10 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
           <t>Julio César Navia</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Puede subir 2-3€ vs. la vez pasada</t>
-        </is>
-      </c>
+      <c r="G9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -853,403 +781,20 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
           <t>Julio César Navia</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Regalo de Levis por encargarles el rótulo luminoso — no requiere aprobación de gasto</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Contenido de las bolsas de provisiones (9 productos)</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Ver detalle abajo</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Ver detalle abajo</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>~356,08€ estimado</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>A definir con Administración</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Marco Guanuchi</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Cantidades faltantes calculadas cruzando contra el inventario oficial — ver hoja "Detalle contenido bolsas"</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL ESTIMADO A ENVIAR</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>≈ 2.833,00€</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Producto</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Stock actual</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Reto 50 hombres</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Faltan</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Compra sugerida</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Precio</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Minis cereal relleno de leche</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C2" t="n">
-        <v>90</v>
-      </c>
-      <c r="D2" t="n">
-        <v>70</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>9 cajas de 8 paq (72u)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>17,55€</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Galletas manzana y avena</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C3" t="n">
-        <v>90</v>
-      </c>
-      <c r="D3" t="n">
-        <v>84</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>11 cajas de 8 paq (88u)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>18,15€</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Galletas choco blanco</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
-        <v>90</v>
-      </c>
-      <c r="D4" t="n">
-        <v>90</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>15 cajas de 6 paq (90u)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>19,50€</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Barras energéticas frutos secos</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>42</v>
-      </c>
-      <c r="C5" t="n">
-        <v>180</v>
-      </c>
-      <c r="D5" t="n">
-        <v>138</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>23 cajas de 6 paq (138u)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>37,95€</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Caramelos surtidos</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2 paquetes</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>5 paquetes</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>A confirmar</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>⚠ Confirmar con Marco Jurado si es el mismo ítem que 'Caramelo Blanco'</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Cola Cao</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>24</v>
-      </c>
-      <c r="C7" t="n">
-        <v>90</v>
-      </c>
-      <c r="D7" t="n">
-        <v>66</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2 cajas de 50 sobres (100u)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>39,98€</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Snickers</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>7</v>
-      </c>
-      <c r="C8" t="n">
-        <v>90</v>
-      </c>
-      <c r="D8" t="n">
-        <v>83</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>17 bolsas de 5u (85u)</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>72,25€</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Sobres Tang</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>10</v>
-      </c>
-      <c r="C9" t="n">
-        <v>90</v>
-      </c>
-      <c r="D9" t="n">
-        <v>80</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>3 cajas de 30u (90u)</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>71,10€</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Fideos Rintin/Maruchan</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>58</v>
-      </c>
-      <c r="C10" t="n">
-        <v>180</v>
-      </c>
-      <c r="D10" t="n">
-        <v>122</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>25 packs de 5 (125u)</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>49,75€</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Atún</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>32</v>
-      </c>
-      <c r="C11" t="n">
-        <v>90</v>
-      </c>
-      <c r="D11" t="n">
-        <v>58</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>15 packs de 4u (60u)</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>29,85€</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL (sin Caramelos, sin resolver)</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>356,08€</t>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>≈ 2.402,91€</t>
         </is>
       </c>
     </row>

</xml_diff>